<commit_message>
Update traffic data 2026-04-17
</commit_message>
<xml_diff>
--- a/CSManager/traffic.xlsx
+++ b/CSManager/traffic.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Views" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clones" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referrers" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Popular Paths" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Downloads" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stats" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Views" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Clones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Referrers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Popular Paths" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Downloads" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Stats" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="9" min="1" max="1"/>
@@ -489,62 +489,62 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="10">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="29" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Total Views</t>
         </is>
       </c>
-      <c r="C1" s="29" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Unique Visitors</t>
         </is>
       </c>
-      <c r="E1" s="29" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="F1" s="29" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Total Views</t>
         </is>
       </c>
-      <c r="G1" s="29" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Unique Visitors</t>
         </is>
       </c>
-      <c r="I1" s="29" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="J1" s="29" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Total Views</t>
         </is>
       </c>
-      <c r="K1" s="29" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Unique Visitors</t>
         </is>
       </c>
-      <c r="M1" s="29" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="N1" s="29" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Total Views</t>
         </is>
       </c>
-      <c r="O1" s="29" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Unique Visitors</t>
         </is>
@@ -553,11 +553,11 @@
     <row r="2" ht="15" customHeight="1" s="10">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C2" t="n">
         <v>2</v>
@@ -568,10 +568,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -579,34 +579,34 @@
         </is>
       </c>
       <c r="J2" t="n">
+        <v>57</v>
+      </c>
+      <c r="K2" t="n">
         <v>32</v>
       </c>
-      <c r="K2" t="n">
-        <v>23</v>
-      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
       <c r="N2" t="n">
+        <v>60</v>
+      </c>
+      <c r="O2" t="n">
         <v>35</v>
-      </c>
-      <c r="O2" t="n">
-        <v>26</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="10">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -634,14 +634,14 @@
     <row r="4" ht="15" customHeight="1" s="10">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -658,14 +658,14 @@
     <row r="5" ht="15" customHeight="1" s="10">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -682,37 +682,37 @@
     <row r="6" ht="15" customHeight="1" s="10">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="10">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="10">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
         <v>3</v>
@@ -721,85 +721,85 @@
     <row r="9" ht="15" customHeight="1" s="10">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="10">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="10">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="10">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="10">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="10">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -812,7 +812,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -825,20 +825,20 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -851,13 +851,52 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" t="n">
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
         <v>1</v>
       </c>
     </row>
@@ -874,7 +913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="9" min="1" max="1"/>
@@ -892,62 +931,62 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="10">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="29" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Total Clones</t>
         </is>
       </c>
-      <c r="C1" s="29" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Unique Cloners</t>
         </is>
       </c>
-      <c r="E1" s="29" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="F1" s="29" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Total Clones</t>
         </is>
       </c>
-      <c r="G1" s="29" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Unique Cloners</t>
         </is>
       </c>
-      <c r="I1" s="29" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="J1" s="29" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Total Clones</t>
         </is>
       </c>
-      <c r="K1" s="29" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Unique Cloners</t>
         </is>
       </c>
-      <c r="M1" s="29" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="N1" s="29" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Total Clones</t>
         </is>
       </c>
-      <c r="O1" s="29" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Unique Cloners</t>
         </is>
@@ -956,14 +995,14 @@
     <row r="2" ht="15" customHeight="1" s="10">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1002,7 +1041,7 @@
     <row r="3" ht="15" customHeight="1" s="10">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1037,7 +1076,7 @@
     <row r="4" ht="15" customHeight="1" s="10">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1061,7 +1100,7 @@
     <row r="5" ht="15" customHeight="1" s="10">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1085,7 +1124,7 @@
     <row r="6" ht="15" customHeight="1" s="10">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1098,7 +1137,7 @@
     <row r="7" ht="15" customHeight="1" s="10">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1111,137 +1150,137 @@
     <row r="8" ht="15" customHeight="1" s="10">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="10">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="10">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-04</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="10">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="10">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="10">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="10">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1254,13 +1293,52 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" t="n">
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1277,7 +1355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:S29"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="9" min="1" max="1"/>
@@ -1299,82 +1377,82 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="10">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date Collected</t>
         </is>
       </c>
-      <c r="B1" s="29" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Referrer</t>
         </is>
       </c>
-      <c r="C1" s="29" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Total Count</t>
         </is>
       </c>
-      <c r="D1" s="29" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="F1" s="29" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="G1" s="29" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Referrer</t>
         </is>
       </c>
-      <c r="H1" s="29" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Total Count</t>
         </is>
       </c>
-      <c r="I1" s="29" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="K1" s="29" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="L1" s="29" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Referrer</t>
         </is>
       </c>
-      <c r="M1" s="29" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Total Count</t>
         </is>
       </c>
-      <c r="N1" s="29" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="P1" s="29" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="Q1" s="29" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Referrer</t>
         </is>
       </c>
-      <c r="R1" s="29" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Total Count</t>
         </is>
       </c>
-      <c r="S1" s="29" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
@@ -1383,7 +1461,7 @@
     <row r="2" ht="15" customHeight="1" s="10">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1392,10 +1470,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1408,10 +1486,10 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="I2" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -1424,10 +1502,10 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>101</v>
+        <v>123</v>
       </c>
       <c r="N2" t="n">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -1440,82 +1518,82 @@
         </is>
       </c>
       <c r="R2" t="n">
-        <v>101</v>
+        <v>123</v>
       </c>
       <c r="S2" t="n">
-        <v>65</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="10">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>github.com</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-W16</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>github.com</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>8</v>
+      </c>
+      <c r="I3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>Bing</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-W16</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="M3" t="n">
+        <v>16</v>
+      </c>
+      <c r="N3" t="n">
+        <v>8</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Bing</t>
         </is>
       </c>
-      <c r="H3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Bing</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>14</v>
-      </c>
-      <c r="N3" t="n">
-        <v>7</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Bing</t>
-        </is>
-      </c>
       <c r="R3" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="S3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="10">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1524,10 +1602,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1536,14 +1614,14 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Bing</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1552,14 +1630,14 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>github.com</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="N4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -1568,29 +1646,29 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>github.com</t>
         </is>
       </c>
       <c r="R4" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="S4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="10">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>github.com</t>
+          <t>Bing</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -1602,14 +1680,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>github.com</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1618,14 +1696,14 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>github.com</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -1634,20 +1712,20 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>github.com</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1656,10 +1734,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1681,19 +1759,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>yseto.net</t>
+          <t>Bing</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1715,19 +1793,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>yseto.net</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1749,19 +1827,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>yseto.net</t>
+          <t>github.com</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1788,14 +1866,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bing</t>
+          <t>yseto.net</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -1806,14 +1884,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bing</t>
+          <t>yseto.net</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -1824,14 +1902,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bing</t>
+          <t>yseto.net</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -1842,14 +1920,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bing</t>
+          <t>yseto.net</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -1860,11 +1938,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Bing</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
@@ -1878,11 +1956,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>github.com</t>
+          <t>Bing</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -1896,11 +1974,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Bing</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -1914,11 +1992,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>github.com</t>
+          <t>Bing</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
@@ -1999,34 +2077,34 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>yseto.net</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Bing</t>
+          <t>github.com</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
         <v>1</v>
@@ -2035,7 +2113,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2053,7 +2131,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2071,7 +2149,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2089,7 +2167,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2107,7 +2185,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2125,18 +2203,90 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>github.com</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>yseto.net</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>11</v>
+      </c>
+      <c r="D30" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Bing</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>github.com</t>
         </is>
       </c>
-      <c r="C29" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" t="n">
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2153,7 +2303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:W29"/>
+  <dimension ref="A1:W39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="9" min="1" max="1"/>
@@ -2179,102 +2329,102 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="10">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date Collected</t>
         </is>
       </c>
-      <c r="B1" s="29" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Path</t>
         </is>
       </c>
-      <c r="C1" s="29" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" s="29" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Total Count</t>
         </is>
       </c>
-      <c r="E1" s="29" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="G1" s="29" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="H1" s="29" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Path</t>
         </is>
       </c>
-      <c r="I1" s="29" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J1" s="29" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Total Count</t>
         </is>
       </c>
-      <c r="K1" s="29" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="M1" s="29" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="N1" s="29" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Path</t>
         </is>
       </c>
-      <c r="O1" s="29" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="P1" s="29" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Total Count</t>
         </is>
       </c>
-      <c r="Q1" s="29" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="S1" s="29" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="T1" s="29" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Path</t>
         </is>
       </c>
-      <c r="U1" s="29" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="V1" s="29" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Total Count</t>
         </is>
       </c>
-      <c r="W1" s="29" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
@@ -2283,7 +2433,7 @@
     <row r="2" ht="15" customHeight="1" s="10">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2297,10 +2447,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E2" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2318,10 +2468,10 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="K2" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -2339,10 +2489,10 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>131</v>
+        <v>162</v>
       </c>
       <c r="Q2" t="n">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -2360,16 +2510,16 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>131</v>
+        <v>162</v>
       </c>
       <c r="W2" t="n">
-        <v>94</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="10">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2383,10 +2533,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2404,10 +2554,10 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -2416,19 +2566,19 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases</t>
+          <t>/seto77/CSManager</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>/releases</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="Q3" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -2437,25 +2587,25 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases</t>
+          <t>/seto77/CSManager</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>/releases</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="W3" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="10">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2469,10 +2619,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2490,10 +2640,10 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -2502,19 +2652,19 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>/seto77/CSManager</t>
+          <t>/seto77/CSManager/releases</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>/releases</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="Q4" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -2523,42 +2673,42 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>/seto77/CSManager</t>
+          <t>/seto77/CSManager/releases</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>/releases</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="W4" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="10">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+          <t>/seto77/CSManager/tree/master/COD</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.909</t>
+          <t>/tree/master/COD</t>
         </is>
       </c>
       <c r="D5" t="n">
         <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2567,19 +2717,19 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+          <t>/seto77/CSManager/tree/master/COD</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.909</t>
+          <t>/tree/master/COD</t>
         </is>
       </c>
       <c r="J5" t="n">
         <v>2</v>
       </c>
       <c r="K5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -2627,262 +2777,619 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.910</t>
+          <t>/seto77/CSManager/blob/master/README.md</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.910</t>
+          <t>/blob/master/README.md</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-W15</t>
+          <t>2026-W16</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.910</t>
+          <t>/seto77/CSManager/releases/tag/v.1.909</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.910</t>
+          <t>/releases/tag/v.1.909</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>106</v>
+        <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>78</v>
+        <v>2</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/tree/master/COD</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>/tree/master/COD</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/tree/master/COD</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>/tree/master/COD</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>2</v>
+      </c>
+      <c r="W6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.910</t>
+          <t>/seto77/CSManager/issues</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.910</t>
+          <t>/issues</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-W15</t>
+          <t>2026-W16</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases</t>
+          <t>/seto77/CSManager/blob/master/README.md</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>/releases</t>
+          <t>/blob/master/README.md</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>23</v>
+        <v>1</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/blob/master/README.md</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>/blob/master/README.md</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/blob/master/README.md</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>/blob/master/README.md</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.910</t>
+          <t>/seto77/CSManager/pulls</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.910</t>
+          <t>/pulls</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-W15</t>
+          <t>2026-W16</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>/seto77/CSManager</t>
+          <t>/seto77/CSManager/issues</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>/issues</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>18</v>
+        <v>1</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/issues</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>/issues</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/issues</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>/issues</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>1</v>
+      </c>
+      <c r="W8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.910</t>
+          <t>/seto77/CSManager/tree/master/COD/COD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.910</t>
+          <t>/tree/master/COD/COD</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-W15</t>
+          <t>2026-W16</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+          <t>/seto77/CSManager/pulls</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.909</t>
+          <t>/pulls</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>12</v>
+        <v>1</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/pulls</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>/pulls</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/pulls</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>/pulls</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>1</v>
+      </c>
+      <c r="W9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases</t>
+          <t>/seto77/CSManager/tree/master/CSManager</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>/releases</t>
+          <t>/tree/master/CSManager</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-W16</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/tree/master/COD/COD</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>/tree/master/COD/COD</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/tree/master/COD/COD</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>/tree/master/COD/COD</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/tree/master/COD/COD</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>/tree/master/COD/COD</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>1</v>
+      </c>
+      <c r="W10" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>/seto77/CSManager</t>
+          <t>/seto77/CSManager/tree/master/CSManager/Properties</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>/tree/master/CSManager/Properties</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-W16</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/tree/master/CSManager</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>/tree/master/CSManager</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/tree/master/CSManager</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>/tree/master/CSManager</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/tree/master/CSManager</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>/tree/master/CSManager</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>1</v>
+      </c>
+      <c r="W11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>/seto77/CSManager</t>
+          <t>/seto77/CSManager/releases/tag/v.1.910</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>/releases/tag/v.1.910</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>16</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-W16</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/tree/master/CSManager/Properties</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>/tree/master/CSManager/Properties</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/tree/master/CSManager/Properties</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>/tree/master/CSManager/Properties</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/tree/master/CSManager/Properties</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>/tree/master/CSManager/Properties</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>1</v>
+      </c>
+      <c r="W12" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases</t>
+          <t>/seto77/CSManager</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>/releases</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -2891,21 +3398,42 @@
       <c r="E13" t="n">
         <v>3</v>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-W15</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/releases/tag/v.1.910</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>/releases/tag/v.1.910</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>106</v>
+      </c>
+      <c r="K13" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/seto77/CSManager</t>
+          <t>/seto77/CSManager/releases</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>/releases</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -2914,28 +3442,70 @@
       <c r="E14" t="n">
         <v>3</v>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-W15</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/releases</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>/releases</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>23</v>
+      </c>
+      <c r="K14" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases</t>
+          <t>/seto77/CSManager/releases/tag/v.1.909</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>/releases</t>
+          <t>/releases/tag/v.1.909</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-W15</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>18</v>
+      </c>
+      <c r="K15" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -2946,19 +3516,40 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/seto77/CSManager</t>
+          <t>/seto77/CSManager/releases/tag/v.1.910</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>/releases/tag/v.1.910</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>14</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-W15</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>/releases/tag/v.1.909</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>12</v>
+      </c>
+      <c r="K16" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -2969,19 +3560,19 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases</t>
+          <t>/seto77/CSManager/releases/tag/v.1.910</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>/releases</t>
+          <t>/releases/tag/v.1.910</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18">
@@ -2992,19 +3583,19 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+          <t>/seto77/CSManager/releases/tag/v.1.910</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.909</t>
+          <t>/releases/tag/v.1.910</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19">
@@ -3015,19 +3606,19 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+          <t>/seto77/CSManager/releases/tag/v.1.910</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.909</t>
+          <t>/releases/tag/v.1.910</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20">
@@ -3038,19 +3629,19 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+          <t>/seto77/CSManager/releases</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.909</t>
+          <t>/releases</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -3061,48 +3652,48 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+          <t>/seto77/CSManager</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.909</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.910</t>
+          <t>/seto77/CSManager</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.910</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3116,16 +3707,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3148,53 +3739,53 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+          <t>/seto77/CSManager/releases</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.909</t>
+          <t>/releases</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>/seto77/CSManager/releases/tag/v.1.910</t>
+          <t>/seto77/CSManager</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>/releases/tag/v.1.910</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3208,55 +3799,285 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>/seto77/CSManager</t>
+          <t>/seto77/CSManager/releases/tag/v.1.909</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>/releases/tag/v.1.909</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>/releases/tag/v.1.909</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>/releases/tag/v.1.909</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>/releases/tag/v.1.909</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/releases/tag/v.1.910</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>/releases/tag/v.1.910</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>15</v>
+      </c>
+      <c r="E32" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/releases</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>/releases</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/releases/tag/v.1.909</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>/releases/tag/v.1.909</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/releases/tag/v.1.910</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>/releases/tag/v.1.910</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>15</v>
+      </c>
+      <c r="E36" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager/releases</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>/releases</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>/seto77/CSManager</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
         <is>
           <t>/seto77/CSManager/releases/tag/v.1.909</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>/releases/tag/v.1.909</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>2</v>
-      </c>
-      <c r="E29" t="n">
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3288,22 +4109,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Release Tag</t>
         </is>
       </c>
-      <c r="B1" s="29" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Release Date</t>
         </is>
       </c>
-      <c r="C1" s="29" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Asset Name</t>
         </is>
       </c>
-      <c r="D1" s="29" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Download Count</t>
         </is>
@@ -3326,7 +4147,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -3950,13 +4771,13 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="30" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D34" s="30" t="n">
-        <v>3924</v>
+      <c r="D34" t="n">
+        <v>3929</v>
       </c>
     </row>
   </sheetData>
@@ -3970,7 +4791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:W5"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="9" min="1" max="1"/>
@@ -3996,102 +4817,102 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="10">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="29" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Stars</t>
         </is>
       </c>
-      <c r="C1" s="29" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Forks</t>
         </is>
       </c>
-      <c r="D1" s="29" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Open Issues</t>
         </is>
       </c>
-      <c r="E1" s="29" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Watchers</t>
         </is>
       </c>
-      <c r="G1" s="29" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="H1" s="29" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Stars</t>
         </is>
       </c>
-      <c r="I1" s="29" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Forks</t>
         </is>
       </c>
-      <c r="J1" s="29" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Open Issues</t>
         </is>
       </c>
-      <c r="K1" s="29" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Watchers</t>
         </is>
       </c>
-      <c r="M1" s="29" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="N1" s="29" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Stars</t>
         </is>
       </c>
-      <c r="O1" s="29" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Forks</t>
         </is>
       </c>
-      <c r="P1" s="29" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Open Issues</t>
         </is>
       </c>
-      <c r="Q1" s="29" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Watchers</t>
         </is>
       </c>
-      <c r="S1" s="29" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="T1" s="29" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Stars</t>
         </is>
       </c>
-      <c r="U1" s="29" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Forks</t>
         </is>
       </c>
-      <c r="V1" s="29" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Open Issues</t>
         </is>
       </c>
-      <c r="W1" s="29" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Watchers</t>
         </is>
@@ -4100,7 +4921,7 @@
     <row r="2" ht="15" customHeight="1" s="10">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -4113,7 +4934,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -4130,7 +4951,7 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -4147,7 +4968,7 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -4164,13 +4985,13 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -4183,7 +5004,7 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -4206,7 +5027,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -4219,13 +5040,13 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -4238,6 +5059,25 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>